<commit_message>
Cattle slurry Print and plots
Created plots and print for the cattle slurry script to make final results quicker to evaluate
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-02-19-pig-slurry/2026-02-19-pig-slurry-picarro.xlsx
+++ b/Lab-trails/2026-02-19-pig-slurry/2026-02-19-pig-slurry-picarro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-02-19-pig-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E8E74C-5405-416F-AE72-959282AE7AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42011724-95C2-4AFA-A1A1-4E9C554DFDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,6 +41,7 @@
     <author>tc={8DC1FA48-6C73-43B8-B575-39BC1BCA9B35}</author>
     <author>tc={41F19D6E-E99D-4BC4-9CF8-03971525C4BB}</author>
     <author>tc={34F919C0-E213-42BB-B018-7CF158825172}</author>
+    <author>tc={9EFC68A0-E0CF-42A9-8A43-AB7809A53DCD}</author>
     <author>tc={BD837BDB-798F-46E2-9B1E-095AD2C34354}</author>
     <author>tc={74A47A3C-9B82-4D0E-8273-A61F47053664}</author>
   </authors>
@@ -71,7 +72,15 @@
     Not exact time - need to go into file and find valve 1 for exact</t>
       </text>
     </comment>
-    <comment ref="F3" authorId="3" shapeId="0" xr:uid="{BD837BDB-798F-46E2-9B1E-095AD2C34354}">
+    <comment ref="M2" authorId="3" shapeId="0" xr:uid="{9EFC68A0-E0CF-42A9-8A43-AB7809A53DCD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Approx time when starting to measure the valves, not the end of the last cycle</t>
+      </text>
+    </comment>
+    <comment ref="F3" authorId="4" shapeId="0" xr:uid="{BD837BDB-798F-46E2-9B1E-095AD2C34354}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +88,7 @@
     The red plastic piece of this one was not replaced with glass</t>
       </text>
     </comment>
-    <comment ref="I14" authorId="4" shapeId="0" xr:uid="{74A47A3C-9B82-4D0E-8273-A61F47053664}">
+    <comment ref="I14" authorId="5" shapeId="0" xr:uid="{74A47A3C-9B82-4D0E-8273-A61F47053664}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -92,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="25">
   <si>
     <t>Valve code</t>
   </si>
@@ -164,6 +173,9 @@
   </si>
   <si>
     <t>02/19-2026</t>
+  </si>
+  <si>
+    <t>02/25-2026</t>
   </si>
 </sst>
 </file>
@@ -531,6 +543,9 @@
   <threadedComment ref="G2" dT="2026-02-22T14:00:45.12" personId="{41FB0084-A38E-4055-BCE6-FE39473376DA}" id="{34F919C0-E213-42BB-B018-7CF158825172}">
     <text>Not exact time - need to go into file and find valve 1 for exact</text>
   </threadedComment>
+  <threadedComment ref="M2" dT="2026-02-26T10:23:52.59" personId="{41FB0084-A38E-4055-BCE6-FE39473376DA}" id="{9EFC68A0-E0CF-42A9-8A43-AB7809A53DCD}">
+    <text>Approx time when starting to measure the valves, not the end of the last cycle</text>
+  </threadedComment>
   <threadedComment ref="F3" dT="2026-02-22T13:48:32.41" personId="{41FB0084-A38E-4055-BCE6-FE39473376DA}" id="{BD837BDB-798F-46E2-9B1E-095AD2C34354}">
     <text>The red plastic piece of this one was not replaced with glass</text>
   </threadedComment>
@@ -552,10 +567,11 @@
     <col min="6" max="7" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -586,10 +602,10 @@
       <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="M1" t="s">
@@ -630,8 +646,18 @@
       <c r="J2">
         <v>0.94899999999999995</v>
       </c>
-      <c r="M2" s="1"/>
-      <c r="N2" s="2"/>
+      <c r="K2" s="3">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="L2" s="3">
+        <v>0.97599999999999998</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0.11874999999999999</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
@@ -656,6 +682,12 @@
       <c r="J3" s="3">
         <v>0.95</v>
       </c>
+      <c r="K3" s="3">
+        <v>0.22</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0.96599999999999997</v>
+      </c>
       <c r="O3" s="6"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -680,6 +712,12 @@
       <c r="J4" s="3">
         <v>0.94699999999999995</v>
       </c>
+      <c r="K4" s="3">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="L4" s="3">
+        <v>0.97499999999999998</v>
+      </c>
       <c r="O4" s="6"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -704,6 +742,12 @@
       <c r="J5">
         <v>0.94699999999999995</v>
       </c>
+      <c r="K5" s="3">
+        <v>0.21099999999999999</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0.97799999999999998</v>
+      </c>
       <c r="O5" s="6"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -728,6 +772,12 @@
       <c r="J6">
         <v>0.94499999999999995</v>
       </c>
+      <c r="K6" s="3">
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="L6" s="3">
+        <v>0.97299999999999998</v>
+      </c>
       <c r="O6" s="6"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -752,6 +802,12 @@
       <c r="J7">
         <v>0.79400000000000004</v>
       </c>
+      <c r="K7" s="3">
+        <v>0.39600000000000002</v>
+      </c>
+      <c r="L7" s="3">
+        <v>0.79500000000000004</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -775,6 +831,12 @@
       <c r="J8" s="3">
         <v>0.94699999999999995</v>
       </c>
+      <c r="K8" s="3">
+        <v>0.216</v>
+      </c>
+      <c r="L8" s="3">
+        <v>0.97</v>
+      </c>
       <c r="O8" s="6"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -799,7 +861,12 @@
       <c r="J9" s="3">
         <v>0.95</v>
       </c>
-      <c r="K9" s="3"/>
+      <c r="K9" s="3">
+        <v>0.217</v>
+      </c>
+      <c r="L9" s="3">
+        <v>0.97</v>
+      </c>
       <c r="O9" s="6"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -824,6 +891,12 @@
       <c r="J10">
         <v>0.94699999999999995</v>
       </c>
+      <c r="K10" s="3">
+        <v>0.217</v>
+      </c>
+      <c r="L10" s="3">
+        <v>0.97</v>
+      </c>
       <c r="O10" s="6"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
@@ -848,6 +921,12 @@
       <c r="J11" s="3">
         <v>0.95</v>
       </c>
+      <c r="K11" s="3">
+        <v>0.218</v>
+      </c>
+      <c r="L11" s="3">
+        <v>0.96799999999999997</v>
+      </c>
       <c r="O11" s="6"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
@@ -872,6 +951,12 @@
       <c r="J12" s="3">
         <v>0.95099999999999996</v>
       </c>
+      <c r="K12" s="3">
+        <v>0.222</v>
+      </c>
+      <c r="L12" s="3">
+        <v>0.96499999999999997</v>
+      </c>
       <c r="O12" s="6"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -893,6 +978,12 @@
       <c r="J13" s="3">
         <v>0.95099999999999996</v>
       </c>
+      <c r="K13" s="3">
+        <v>0.39700000000000002</v>
+      </c>
+      <c r="L13" s="3">
+        <v>0.79600000000000004</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
@@ -918,7 +1009,12 @@
         <f>AVERAGE(J7,J20,J25)</f>
         <v>0.76833333333333342</v>
       </c>
-      <c r="K14" s="3"/>
+      <c r="K14" s="3">
+        <v>0.223</v>
+      </c>
+      <c r="L14" s="3">
+        <v>0.95399999999999996</v>
+      </c>
       <c r="O14" s="6"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
@@ -943,6 +1039,12 @@
       <c r="J15" s="3">
         <v>0.95099999999999996</v>
       </c>
+      <c r="K15" s="3">
+        <v>0.20899999999999999</v>
+      </c>
+      <c r="L15" s="3">
+        <v>0.97799999999999998</v>
+      </c>
       <c r="O15" s="6"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
@@ -967,6 +1069,12 @@
       <c r="J16" s="3">
         <v>0.95099999999999996</v>
       </c>
+      <c r="K16" s="3">
+        <v>0.192</v>
+      </c>
+      <c r="L16" s="3">
+        <v>0.99399999999999999</v>
+      </c>
       <c r="O16" s="6"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
@@ -991,6 +1099,12 @@
       <c r="J17" s="3">
         <v>0.94899999999999995</v>
       </c>
+      <c r="K17" s="3">
+        <v>0.215</v>
+      </c>
+      <c r="L17" s="3">
+        <v>0.97199999999999998</v>
+      </c>
       <c r="O17" s="6"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
@@ -1015,6 +1129,12 @@
       <c r="J18" s="3">
         <v>0.94599999999999995</v>
       </c>
+      <c r="K18" s="3">
+        <v>0.22</v>
+      </c>
+      <c r="L18" s="3">
+        <v>0.96699999999999997</v>
+      </c>
       <c r="O18" s="6"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
@@ -1039,6 +1159,12 @@
       <c r="J19" s="3">
         <v>0.95</v>
       </c>
+      <c r="K19" s="3">
+        <v>0.752</v>
+      </c>
+      <c r="L19" s="3">
+        <v>0.439</v>
+      </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20">
@@ -1062,6 +1188,12 @@
       <c r="J20" s="3">
         <v>0.75600000000000001</v>
       </c>
+      <c r="K20" s="3">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="L20" s="3">
+        <v>0.97399999999999998</v>
+      </c>
       <c r="O20" s="6"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
@@ -1086,6 +1218,12 @@
       <c r="J21" s="3">
         <v>0.95</v>
       </c>
+      <c r="K21" s="3">
+        <v>0.224</v>
+      </c>
+      <c r="L21" s="3">
+        <v>0.96499999999999997</v>
+      </c>
       <c r="O21" s="6"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
@@ -1110,6 +1248,12 @@
       <c r="J22" s="3">
         <v>0.94899999999999995</v>
       </c>
+      <c r="K22" s="3">
+        <v>0.20899999999999999</v>
+      </c>
+      <c r="L22" s="3">
+        <v>0.97899999999999998</v>
+      </c>
       <c r="O22" s="6"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
@@ -1134,6 +1278,12 @@
       <c r="J23" s="3">
         <v>0.95</v>
       </c>
+      <c r="K23" s="3">
+        <v>0.22700000000000001</v>
+      </c>
+      <c r="L23" s="3">
+        <v>0.96099999999999997</v>
+      </c>
       <c r="O23" s="6"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
@@ -1158,6 +1308,12 @@
       <c r="J24" s="3">
         <v>0.94799999999999995</v>
       </c>
+      <c r="K24" s="3">
+        <v>0.21099999999999999</v>
+      </c>
+      <c r="L24" s="3">
+        <v>0.97599999999999998</v>
+      </c>
       <c r="O24" s="6"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -1178,6 +1334,12 @@
       </c>
       <c r="J25" s="3">
         <v>0.755</v>
+      </c>
+      <c r="K25" s="3">
+        <v>0.441</v>
+      </c>
+      <c r="L25" s="3">
+        <v>0.753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>